<commit_message>
Removed database to reduce size before commit
Debugged stockpile profile report
</commit_message>
<xml_diff>
--- a/blendmaster_OOP/output/optimised_blend_report_2024-11-28_06-00.xlsx
+++ b/blendmaster_OOP/output/optimised_blend_report_2024-11-28_06-00.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL16"/>
+  <dimension ref="A1:AL33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,7 +629,7 @@
         <v>45624.25</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45624.54549155224</v>
+        <v>45624.26702842084</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -641,7 +641,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>7.091797253888889</v>
+        <v>0.4086820999999999</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -650,35 +650,35 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0104</t>
+          <t>ELW01_RP01_0212</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>0.33</v>
+        <v>0.26</v>
       </c>
       <c r="J2" t="n">
-        <v>373527.772</v>
+        <v>225234.6115</v>
       </c>
       <c r="K2" t="n">
-        <v>7091.797253888889</v>
+        <v>322.5298876333841</v>
       </c>
       <c r="L2" t="n">
-        <v>366435.9747461111</v>
+        <v>224912.0816123666</v>
       </c>
       <c r="M2" t="n">
-        <v>61.30134911866624</v>
+        <v>60.52178373729767</v>
       </c>
       <c r="N2" t="n">
-        <v>3.879912510809882</v>
+        <v>4.059457898875317</v>
       </c>
       <c r="O2" t="n">
-        <v>2.568357585519593</v>
+        <v>3.033311423801729</v>
       </c>
       <c r="P2" t="n">
-        <v>0.1208336982910231</v>
+        <v>0.1912254150327387</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.04347089716331926</v>
+        <v>0.04966826077403921</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -689,10 +689,10 @@
         <v>1000</v>
       </c>
       <c r="T2" t="n">
-        <v>1000</v>
+        <v>789.1950433683886</v>
       </c>
       <c r="U2" t="n">
-        <v>21275.39176166667</v>
+        <v>1226.0463</v>
       </c>
       <c r="V2" t="n">
         <v>3000</v>
@@ -701,25 +701,25 @@
         <v>3000</v>
       </c>
       <c r="X2" t="n">
-        <v>60.89230864367209</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="Y2" t="n">
-        <v>4.347718101919434</v>
+        <v>6.098594256090682</v>
       </c>
       <c r="Z2" t="n">
-        <v>2.414439256130773</v>
+        <v>3.868554741238664</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.1184842652498511</v>
+        <v>0.1145784485168504</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.0370920044818143</v>
+        <v>0.04956257802280711</v>
       </c>
       <c r="AC2" t="n">
         <v>58</v>
       </c>
       <c r="AD2" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
@@ -751,7 +751,7 @@
         <v>45624.25</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45624.54549155224</v>
+        <v>45624.26702842084</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -763,7 +763,7 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>7.091797253888889</v>
+        <v>0.4086820999999999</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -772,35 +772,35 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0105</t>
+          <t>FLY01_RP01_0801</t>
         </is>
       </c>
       <c r="I3" t="n">
         <v>0.33</v>
       </c>
       <c r="J3" t="n">
-        <v>236195.31475</v>
+        <v>408.6820999999999</v>
       </c>
       <c r="K3" t="n">
-        <v>7091.797253888889</v>
+        <v>408.6820999999999</v>
       </c>
       <c r="L3" t="n">
-        <v>229103.5174961111</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>59.58008479807087</v>
+        <v>55.56862076349383</v>
       </c>
       <c r="N3" t="n">
-        <v>5.253888040550701</v>
+        <v>4.715978440440851</v>
       </c>
       <c r="O3" t="n">
-        <v>2.368739705797716</v>
+        <v>5.580065987524456</v>
       </c>
       <c r="P3" t="n">
-        <v>0.1124777124620528</v>
+        <v>0.05066384624236227</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.03174950411324488</v>
+        <v>0.02174606032201762</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
         <v>1000</v>
       </c>
       <c r="U3" t="n">
-        <v>21275.39176166667</v>
+        <v>1226.0463</v>
       </c>
       <c r="V3" t="n">
         <v>3000</v>
@@ -823,25 +823,25 @@
         <v>3000</v>
       </c>
       <c r="X3" t="n">
-        <v>60.89230864367209</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="Y3" t="n">
-        <v>4.347718101919434</v>
+        <v>6.098594256090682</v>
       </c>
       <c r="Z3" t="n">
-        <v>2.414439256130773</v>
+        <v>3.868554741238664</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.1184842652498511</v>
+        <v>0.1145784485168504</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.0370920044818143</v>
+        <v>0.04956257802280711</v>
       </c>
       <c r="AC3" t="n">
         <v>58</v>
       </c>
       <c r="AD3" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE3" t="n">
         <v>0</v>
@@ -873,7 +873,7 @@
         <v>45624.25</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45624.54549155224</v>
+        <v>45624.26702842084</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -885,7 +885,7 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>7.091797253888889</v>
+        <v>0.4086820999999999</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -894,35 +894,35 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0109</t>
+          <t>WED01_RP01_0703</t>
         </is>
       </c>
       <c r="I4" t="n">
         <v>0.33</v>
       </c>
       <c r="J4" t="n">
-        <v>363724.09875</v>
+        <v>1813.5</v>
       </c>
       <c r="K4" t="n">
-        <v>7091.797253888889</v>
+        <v>408.6820999999999</v>
       </c>
       <c r="L4" t="n">
-        <v>356632.3014961111</v>
+        <v>1404.8179</v>
       </c>
       <c r="M4" t="n">
-        <v>61.79549201427914</v>
+        <v>62.11737649943012</v>
       </c>
       <c r="N4" t="n">
-        <v>3.909353754397719</v>
+        <v>3.134631429873529</v>
       </c>
       <c r="O4" t="n">
-        <v>2.306220477075012</v>
+        <v>3.090828380605592</v>
       </c>
       <c r="P4" t="n">
-        <v>0.1221413849964776</v>
+        <v>0.1197800917964288</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.03605561216887876</v>
+        <v>0.05543724900208404</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -936,7 +936,7 @@
         <v>1000</v>
       </c>
       <c r="U4" t="n">
-        <v>21275.39176166667</v>
+        <v>1226.0463</v>
       </c>
       <c r="V4" t="n">
         <v>3000</v>
@@ -945,25 +945,25 @@
         <v>3000</v>
       </c>
       <c r="X4" t="n">
-        <v>60.89230864367209</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="Y4" t="n">
-        <v>4.347718101919434</v>
+        <v>6.098594256090682</v>
       </c>
       <c r="Z4" t="n">
-        <v>2.414439256130773</v>
+        <v>3.868554741238664</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.1184842652498511</v>
+        <v>0.1145784485168504</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.0370920044818143</v>
+        <v>0.04956257802280711</v>
       </c>
       <c r="AC4" t="n">
         <v>58</v>
       </c>
       <c r="AD4" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
@@ -992,13 +992,13 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45624.54549155224</v>
+        <v>45624.25</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45624.68828857363</v>
+        <v>45624.26702842084</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
@@ -1007,7 +1007,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>3.427128513333333</v>
+        <v>0.4086820999999999</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1016,35 +1016,35 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0104</t>
+          <t>WES01_LT01_0901</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>0.33</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>366435.9747461111</v>
+        <v>22141.10000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>3427.128513333334</v>
+        <v>86.1522123666158</v>
       </c>
       <c r="L5" t="n">
-        <v>363008.8462327778</v>
+        <v>22054.94778763339</v>
       </c>
       <c r="M5" t="n">
-        <v>61.30134911866624</v>
+        <v>40.56124264065325</v>
       </c>
       <c r="N5" t="n">
-        <v>3.879912510809882</v>
+        <v>34.35151127901289</v>
       </c>
       <c r="O5" t="n">
-        <v>2.568357585519593</v>
+        <v>2.56585767038744</v>
       </c>
       <c r="P5" t="n">
-        <v>0.1208336982910231</v>
+        <v>0.1061514784064821</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.04347089716331926</v>
+        <v>0.15325294075118</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -1055,10 +1055,10 @@
         <v>1000</v>
       </c>
       <c r="T5" t="n">
-        <v>1000</v>
+        <v>210.8049566316112</v>
       </c>
       <c r="U5" t="n">
-        <v>10281.38554</v>
+        <v>1226.0463</v>
       </c>
       <c r="V5" t="n">
         <v>3000</v>
@@ -1067,25 +1067,25 @@
         <v>3000</v>
       </c>
       <c r="X5" t="n">
-        <v>60.89230864367209</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="Y5" t="n">
-        <v>4.347718101919428</v>
+        <v>6.098594256090682</v>
       </c>
       <c r="Z5" t="n">
-        <v>2.414439256130767</v>
+        <v>3.868554741238664</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.118484265249851</v>
+        <v>0.1145784485168504</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.03709200448181412</v>
+        <v>0.04956257802280711</v>
       </c>
       <c r="AC5" t="n">
         <v>58</v>
       </c>
       <c r="AD5" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
@@ -1114,10 +1114,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45624.54549155224</v>
+        <v>45624.26702842084</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45624.68828857363</v>
+        <v>45624.3255625</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
@@ -1126,10 +1126,10 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>3.427128513333333</v>
+        <v>1.4048179</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1138,35 +1138,35 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0105</t>
+          <t>CEN01_RP01_0109</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>0.33</v>
+        <v>0.03</v>
       </c>
       <c r="J6" t="n">
-        <v>229103.5174961111</v>
+        <v>363724.09875</v>
       </c>
       <c r="K6" t="n">
-        <v>3427.128513333334</v>
+        <v>143.66747301729</v>
       </c>
       <c r="L6" t="n">
-        <v>225676.3889827777</v>
+        <v>363580.4312769827</v>
       </c>
       <c r="M6" t="n">
-        <v>59.58008479807087</v>
+        <v>61.79549201427914</v>
       </c>
       <c r="N6" t="n">
-        <v>5.253888040550701</v>
+        <v>3.909353754397719</v>
       </c>
       <c r="O6" t="n">
-        <v>2.368739705797716</v>
+        <v>2.306220477075012</v>
       </c>
       <c r="P6" t="n">
-        <v>0.1124777124620528</v>
+        <v>0.1221413849964776</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.03174950411324488</v>
+        <v>0.03605561216887876</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1177,10 +1177,10 @@
         <v>1000</v>
       </c>
       <c r="T6" t="n">
-        <v>1000</v>
+        <v>102.2676839591024</v>
       </c>
       <c r="U6" t="n">
-        <v>10281.38554</v>
+        <v>4214.4537</v>
       </c>
       <c r="V6" t="n">
         <v>3000</v>
@@ -1189,25 +1189,25 @@
         <v>3000</v>
       </c>
       <c r="X6" t="n">
-        <v>60.89230864367209</v>
+        <v>58.00000000000001</v>
       </c>
       <c r="Y6" t="n">
-        <v>4.347718101919428</v>
+        <v>6.019595554336112</v>
       </c>
       <c r="Z6" t="n">
-        <v>2.414439256130767</v>
+        <v>4.115528309395112</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.118484265249851</v>
+        <v>0.1166994619512664</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.03709200448181412</v>
+        <v>0.04877589831351777</v>
       </c>
       <c r="AC6" t="n">
         <v>58</v>
       </c>
       <c r="AD6" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE6" t="n">
         <v>0</v>
@@ -1236,10 +1236,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45624.54549155224</v>
+        <v>45624.26702842084</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45624.68828857363</v>
+        <v>45624.3255625</v>
       </c>
       <c r="C7" t="n">
         <v>1</v>
@@ -1248,10 +1248,10 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>3.427128513333333</v>
+        <v>1.4048179</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1260,35 +1260,35 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0109</t>
+          <t>ELW01_LT01_2001</t>
         </is>
       </c>
       <c r="I7" t="n">
         <v>0.33</v>
       </c>
       <c r="J7" t="n">
-        <v>356632.3014961111</v>
+        <v>1048985.1</v>
       </c>
       <c r="K7" t="n">
-        <v>3427.128513333334</v>
+        <v>1404.8179</v>
       </c>
       <c r="L7" t="n">
-        <v>353205.1729827778</v>
+        <v>1047580.2821</v>
       </c>
       <c r="M7" t="n">
-        <v>61.79549201427914</v>
+        <v>56.26801388728946</v>
       </c>
       <c r="N7" t="n">
-        <v>3.909353754397719</v>
+        <v>6.935902734745083</v>
       </c>
       <c r="O7" t="n">
-        <v>2.306220477075012</v>
+        <v>4.976544911650335</v>
       </c>
       <c r="P7" t="n">
-        <v>0.1221413849964776</v>
+        <v>0.1237568390236727</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.03605561216887876</v>
+        <v>0.05754207494577221</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1302,7 +1302,7 @@
         <v>1000</v>
       </c>
       <c r="U7" t="n">
-        <v>10281.38554</v>
+        <v>4214.4537</v>
       </c>
       <c r="V7" t="n">
         <v>3000</v>
@@ -1311,25 +1311,25 @@
         <v>3000</v>
       </c>
       <c r="X7" t="n">
-        <v>60.89230864367209</v>
+        <v>58.00000000000001</v>
       </c>
       <c r="Y7" t="n">
-        <v>4.347718101919428</v>
+        <v>6.019595554336112</v>
       </c>
       <c r="Z7" t="n">
-        <v>2.414439256130767</v>
+        <v>4.115528309395112</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.118484265249851</v>
+        <v>0.1166994619512664</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.03709200448181412</v>
+        <v>0.04877589831351777</v>
       </c>
       <c r="AC7" t="n">
         <v>58</v>
       </c>
       <c r="AD7" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE7" t="n">
         <v>0</v>
@@ -1358,13 +1358,13 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45624.68828857363</v>
+        <v>45624.26702842084</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45624.75</v>
+        <v>45624.3255625</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -1373,7 +1373,7 @@
         <v>2</v>
       </c>
       <c r="F8" t="n">
-        <v>1.481074232777778</v>
+        <v>1.4048179</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1382,35 +1382,35 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0104</t>
+          <t>WED01_RP01_0703</t>
         </is>
       </c>
       <c r="I8" t="n">
         <v>0.33</v>
       </c>
       <c r="J8" t="n">
-        <v>363008.8462327778</v>
+        <v>1404.8179</v>
       </c>
       <c r="K8" t="n">
-        <v>1481.074232777778</v>
+        <v>1404.8179</v>
       </c>
       <c r="L8" t="n">
-        <v>361527.772</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>61.30134911866624</v>
+        <v>62.11737649943012</v>
       </c>
       <c r="N8" t="n">
-        <v>3.879912510809882</v>
+        <v>3.134631429873529</v>
       </c>
       <c r="O8" t="n">
-        <v>2.568357585519593</v>
+        <v>3.090828380605592</v>
       </c>
       <c r="P8" t="n">
-        <v>0.1208336982910231</v>
+        <v>0.1197800917964288</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.04347089716331926</v>
+        <v>0.05543724900208404</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
         <v>1000</v>
       </c>
       <c r="U8" t="n">
-        <v>4443.222698333333</v>
+        <v>4214.4537</v>
       </c>
       <c r="V8" t="n">
         <v>3000</v>
@@ -1433,25 +1433,25 @@
         <v>3000</v>
       </c>
       <c r="X8" t="n">
-        <v>59.71739163763709</v>
+        <v>58.00000000000001</v>
       </c>
       <c r="Y8" t="n">
-        <v>4.558844833296899</v>
+        <v>6.019595554336112</v>
       </c>
       <c r="Z8" t="n">
-        <v>2.706464506200421</v>
+        <v>4.115528309395112</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.1130477991935698</v>
+        <v>0.1166994619512664</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.03716841715414343</v>
+        <v>0.04877589831351777</v>
       </c>
       <c r="AC8" t="n">
         <v>58</v>
       </c>
       <c r="AD8" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE8" t="n">
         <v>0</v>
@@ -1480,13 +1480,13 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45624.68828857363</v>
+        <v>45624.26702842084</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45624.75</v>
+        <v>45624.3255625</v>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
@@ -1495,7 +1495,7 @@
         <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>1.481074232777778</v>
+        <v>1.4048179</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1504,35 +1504,35 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0105</t>
+          <t>WES01_LT01_2001</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>0.33</v>
+        <v>0.3</v>
       </c>
       <c r="J9" t="n">
-        <v>225676.3889827777</v>
+        <v>714322.3000000004</v>
       </c>
       <c r="K9" t="n">
-        <v>1481.074232777778</v>
+        <v>1261.15042698271</v>
       </c>
       <c r="L9" t="n">
-        <v>224195.31475</v>
+        <v>713061.1495730177</v>
       </c>
       <c r="M9" t="n">
-        <v>59.58008479807087</v>
+        <v>54.91049713266775</v>
       </c>
       <c r="N9" t="n">
-        <v>5.253888040550701</v>
+        <v>8.452911640316779</v>
       </c>
       <c r="O9" t="n">
-        <v>2.368739705797716</v>
+        <v>4.503970433939116</v>
       </c>
       <c r="P9" t="n">
-        <v>0.1124777124620528</v>
+        <v>0.1047866238005244</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.03174950411324488</v>
+        <v>0.03303996805335782</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -1543,10 +1543,10 @@
         <v>1000</v>
       </c>
       <c r="T9" t="n">
-        <v>1000</v>
+        <v>897.7323160408976</v>
       </c>
       <c r="U9" t="n">
-        <v>4443.222698333333</v>
+        <v>4214.4537</v>
       </c>
       <c r="V9" t="n">
         <v>3000</v>
@@ -1555,25 +1555,25 @@
         <v>3000</v>
       </c>
       <c r="X9" t="n">
-        <v>59.71739163763709</v>
+        <v>58.00000000000001</v>
       </c>
       <c r="Y9" t="n">
-        <v>4.558844833296899</v>
+        <v>6.019595554336112</v>
       </c>
       <c r="Z9" t="n">
-        <v>2.706464506200421</v>
+        <v>4.115528309395112</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.1130477991935698</v>
+        <v>0.1166994619512664</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.03716841715414343</v>
+        <v>0.04877589831351777</v>
       </c>
       <c r="AC9" t="n">
         <v>58</v>
       </c>
       <c r="AD9" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE9" t="n">
         <v>0</v>
@@ -1602,10 +1602,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45624.68828857363</v>
+        <v>45624.3255625</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45624.75</v>
+        <v>45624.54549155224</v>
       </c>
       <c r="C10" t="n">
         <v>2</v>
@@ -1614,10 +1614,10 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>1.481074232777778</v>
+        <v>5.278297253888889</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1626,35 +1626,35 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0108</t>
+          <t>CEN01_RP01_0105</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>0.33</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>48678.46251805</v>
+        <v>236195.31475</v>
       </c>
       <c r="K10" t="n">
-        <v>1481.074232777778</v>
+        <v>1159.742006133012</v>
       </c>
       <c r="L10" t="n">
-        <v>47197.38828527222</v>
+        <v>235035.5727438669</v>
       </c>
       <c r="M10" t="n">
-        <v>58.27074099617414</v>
+        <v>59.58008479807087</v>
       </c>
       <c r="N10" t="n">
-        <v>4.542733948530114</v>
+        <v>5.253888040550701</v>
       </c>
       <c r="O10" t="n">
-        <v>3.182296227283953</v>
+        <v>2.368739705797716</v>
       </c>
       <c r="P10" t="n">
-        <v>0.1058319868276335</v>
+        <v>0.1124777124620528</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.03628485018586616</v>
+        <v>0.03174950411324488</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>1000</v>
       </c>
       <c r="T10" t="n">
-        <v>1000</v>
+        <v>219.7189643456608</v>
       </c>
       <c r="U10" t="n">
-        <v>4443.222698333333</v>
+        <v>15834.89176166667</v>
       </c>
       <c r="V10" t="n">
         <v>3000</v>
@@ -1677,25 +1677,25 @@
         <v>3000</v>
       </c>
       <c r="X10" t="n">
-        <v>59.71739163763709</v>
+        <v>58</v>
       </c>
       <c r="Y10" t="n">
-        <v>4.558844833296899</v>
+        <v>6.198427325733884</v>
       </c>
       <c r="Z10" t="n">
-        <v>2.706464506200421</v>
+        <v>3.772528379479401</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.1130477991935698</v>
+        <v>0.1174582419520254</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.03716841715414343</v>
+        <v>0.04211803858918725</v>
       </c>
       <c r="AC10" t="n">
         <v>58</v>
       </c>
       <c r="AD10" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE10" t="n">
         <v>0</v>
@@ -1724,13 +1724,13 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45624.75</v>
+        <v>45624.3255625</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45625.25</v>
+        <v>45624.54549155224</v>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -1739,44 +1739,44 @@
         <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>12</v>
+        <v>5.278297253888889</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>period_1</t>
+          <t>preplan</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0104</t>
+          <t>CEN01_RP01_0109</t>
         </is>
       </c>
       <c r="I11" t="n">
         <v>0.33</v>
       </c>
       <c r="J11" t="n">
-        <v>361527.772</v>
+        <v>363580.4312769827</v>
       </c>
       <c r="K11" t="n">
-        <v>12000</v>
+        <v>5278.297253888889</v>
       </c>
       <c r="L11" t="n">
-        <v>349527.772</v>
+        <v>358302.1340230938</v>
       </c>
       <c r="M11" t="n">
-        <v>61.30134911866624</v>
+        <v>61.79549201427914</v>
       </c>
       <c r="N11" t="n">
-        <v>3.879912510809882</v>
+        <v>3.909353754397719</v>
       </c>
       <c r="O11" t="n">
-        <v>2.568357585519593</v>
+        <v>2.306220477075012</v>
       </c>
       <c r="P11" t="n">
-        <v>0.1208336982910231</v>
+        <v>0.1221413849964776</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.04347089716331926</v>
+        <v>0.03605561216887876</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -1790,7 +1790,7 @@
         <v>1000</v>
       </c>
       <c r="U11" t="n">
-        <v>36000</v>
+        <v>15834.89176166667</v>
       </c>
       <c r="V11" t="n">
         <v>3000</v>
@@ -1799,25 +1799,25 @@
         <v>3000</v>
       </c>
       <c r="X11" t="n">
-        <v>59.71739163763709</v>
+        <v>58</v>
       </c>
       <c r="Y11" t="n">
-        <v>4.558844833296899</v>
+        <v>6.198427325733884</v>
       </c>
       <c r="Z11" t="n">
-        <v>2.70646450620042</v>
+        <v>3.772528379479401</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.1130477991935698</v>
+        <v>0.1174582419520254</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.03716841715414343</v>
+        <v>0.04211803858918725</v>
       </c>
       <c r="AC11" t="n">
         <v>58</v>
       </c>
       <c r="AD11" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE11" t="n">
         <v>0</v>
@@ -1846,13 +1846,13 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>45624.75</v>
+        <v>45624.3255625</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45625.25</v>
+        <v>45624.54549155224</v>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -1861,44 +1861,44 @@
         <v>3</v>
       </c>
       <c r="F12" t="n">
-        <v>12</v>
+        <v>5.278297253888889</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>period_1</t>
+          <t>preplan</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0105</t>
+          <t>ELW01_LT01_2001</t>
         </is>
       </c>
       <c r="I12" t="n">
         <v>0.33</v>
       </c>
       <c r="J12" t="n">
-        <v>224195.31475</v>
+        <v>1047580.2821</v>
       </c>
       <c r="K12" t="n">
-        <v>12000</v>
+        <v>5278.297253888889</v>
       </c>
       <c r="L12" t="n">
-        <v>212195.31475</v>
+        <v>1042301.984846111</v>
       </c>
       <c r="M12" t="n">
-        <v>59.58008479807087</v>
+        <v>56.26801388728946</v>
       </c>
       <c r="N12" t="n">
-        <v>5.253888040550701</v>
+        <v>6.935902734745083</v>
       </c>
       <c r="O12" t="n">
-        <v>2.368739705797716</v>
+        <v>4.976544911650335</v>
       </c>
       <c r="P12" t="n">
-        <v>0.1124777124620528</v>
+        <v>0.1237568390236727</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.03174950411324488</v>
+        <v>0.05754207494577221</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -1912,7 +1912,7 @@
         <v>1000</v>
       </c>
       <c r="U12" t="n">
-        <v>36000</v>
+        <v>15834.89176166667</v>
       </c>
       <c r="V12" t="n">
         <v>3000</v>
@@ -1921,25 +1921,25 @@
         <v>3000</v>
       </c>
       <c r="X12" t="n">
-        <v>59.71739163763709</v>
+        <v>58</v>
       </c>
       <c r="Y12" t="n">
-        <v>4.558844833296899</v>
+        <v>6.198427325733884</v>
       </c>
       <c r="Z12" t="n">
-        <v>2.70646450620042</v>
+        <v>3.772528379479401</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.1130477991935698</v>
+        <v>0.1174582419520254</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.03716841715414343</v>
+        <v>0.04211803858918725</v>
       </c>
       <c r="AC12" t="n">
         <v>58</v>
       </c>
       <c r="AD12" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE12" t="n">
         <v>0</v>
@@ -1968,13 +1968,13 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>45624.75</v>
+        <v>45624.3255625</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>45625.25</v>
+        <v>45624.54549155224</v>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
@@ -1983,44 +1983,44 @@
         <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>12</v>
+        <v>5.278297253888889</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>period_1</t>
+          <t>preplan</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0108</t>
+          <t>WES01_LT01_2001</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>0.33</v>
+        <v>0.26</v>
       </c>
       <c r="J13" t="n">
-        <v>47345.61978727223</v>
+        <v>713061.1495730177</v>
       </c>
       <c r="K13" t="n">
-        <v>12000</v>
+        <v>4118.555247755876</v>
       </c>
       <c r="L13" t="n">
-        <v>35345.61978727223</v>
+        <v>708942.5943252619</v>
       </c>
       <c r="M13" t="n">
-        <v>58.27074099617414</v>
+        <v>54.91049713266775</v>
       </c>
       <c r="N13" t="n">
-        <v>4.542733948530114</v>
+        <v>8.452911640316779</v>
       </c>
       <c r="O13" t="n">
-        <v>3.182296227283953</v>
+        <v>4.503970433939116</v>
       </c>
       <c r="P13" t="n">
-        <v>0.1058319868276335</v>
+        <v>0.1047866238005244</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.03628485018586616</v>
+        <v>0.03303996805335782</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -2031,10 +2031,10 @@
         <v>1000</v>
       </c>
       <c r="T13" t="n">
-        <v>1000</v>
+        <v>780.281035654339</v>
       </c>
       <c r="U13" t="n">
-        <v>36000</v>
+        <v>15834.89176166667</v>
       </c>
       <c r="V13" t="n">
         <v>3000</v>
@@ -2043,25 +2043,25 @@
         <v>3000</v>
       </c>
       <c r="X13" t="n">
-        <v>59.71739163763709</v>
+        <v>58</v>
       </c>
       <c r="Y13" t="n">
-        <v>4.558844833296899</v>
+        <v>6.198427325733884</v>
       </c>
       <c r="Z13" t="n">
-        <v>2.70646450620042</v>
+        <v>3.772528379479401</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.1130477991935698</v>
+        <v>0.1174582419520254</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.03716841715414343</v>
+        <v>0.04211803858918725</v>
       </c>
       <c r="AC13" t="n">
         <v>58</v>
       </c>
       <c r="AD13" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE13" t="n">
         <v>0</v>
@@ -2090,59 +2090,59 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>45625.25</v>
+        <v>45624.54549155224</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>45625.75</v>
+        <v>45624.68828857363</v>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F14" t="n">
-        <v>12</v>
+        <v>3.427128513333333</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>period_2</t>
+          <t>preplan</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0104</t>
+          <t>CEN01_RP01_0105</t>
         </is>
       </c>
       <c r="I14" t="n">
         <v>0.33</v>
       </c>
       <c r="J14" t="n">
-        <v>349527.772</v>
+        <v>235035.5727438669</v>
       </c>
       <c r="K14" t="n">
-        <v>12000</v>
+        <v>3427.128513333334</v>
       </c>
       <c r="L14" t="n">
-        <v>337527.772</v>
+        <v>231608.4442305336</v>
       </c>
       <c r="M14" t="n">
-        <v>61.30134911866624</v>
+        <v>59.58008479807087</v>
       </c>
       <c r="N14" t="n">
-        <v>3.879912510809882</v>
+        <v>5.253888040550701</v>
       </c>
       <c r="O14" t="n">
-        <v>2.568357585519593</v>
+        <v>2.368739705797716</v>
       </c>
       <c r="P14" t="n">
-        <v>0.1208336982910231</v>
+        <v>0.1124777124620528</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.04347089716331926</v>
+        <v>0.03174950411324488</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -2156,7 +2156,7 @@
         <v>1000</v>
       </c>
       <c r="U14" t="n">
-        <v>36000</v>
+        <v>10281.38554</v>
       </c>
       <c r="V14" t="n">
         <v>3000</v>
@@ -2165,25 +2165,25 @@
         <v>3000</v>
       </c>
       <c r="X14" t="n">
-        <v>59.71739163763709</v>
+        <v>58.00000000000001</v>
       </c>
       <c r="Y14" t="n">
-        <v>4.558844833296899</v>
+        <v>6.340414684271129</v>
       </c>
       <c r="Z14" t="n">
-        <v>2.70646450620042</v>
+        <v>2.925925826310943</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.1130477991935698</v>
+        <v>0.108383693596484</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.03716841715414343</v>
+        <v>0.07492946116501936</v>
       </c>
       <c r="AC14" t="n">
         <v>58</v>
       </c>
       <c r="AD14" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE14" t="n">
         <v>0</v>
@@ -2212,59 +2212,59 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>45625.25</v>
+        <v>45624.54549155224</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>45625.75</v>
+        <v>45624.68828857363</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F15" t="n">
-        <v>12</v>
+        <v>3.427128513333333</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>period_2</t>
+          <t>preplan</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0105</t>
+          <t>ELW01_RP01_0807</t>
         </is>
       </c>
       <c r="I15" t="n">
         <v>0.33</v>
       </c>
       <c r="J15" t="n">
-        <v>212195.31475</v>
+        <v>13191.616</v>
       </c>
       <c r="K15" t="n">
-        <v>12000</v>
+        <v>3370.281110881937</v>
       </c>
       <c r="L15" t="n">
-        <v>200195.31475</v>
+        <v>9821.334889118063</v>
       </c>
       <c r="M15" t="n">
-        <v>59.58008479807087</v>
+        <v>59.57843439126294</v>
       </c>
       <c r="N15" t="n">
-        <v>5.253888040550701</v>
+        <v>4.225669895284223</v>
       </c>
       <c r="O15" t="n">
-        <v>2.368739705797716</v>
+        <v>2.502769386280923</v>
       </c>
       <c r="P15" t="n">
-        <v>0.1124777124620528</v>
+        <v>0.1068578171766122</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.03174950411324488</v>
+        <v>0.03796622173938611</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -2275,10 +2275,10 @@
         <v>1000</v>
       </c>
       <c r="T15" t="n">
-        <v>1000</v>
+        <v>983.4125267756287</v>
       </c>
       <c r="U15" t="n">
-        <v>36000</v>
+        <v>10281.38554</v>
       </c>
       <c r="V15" t="n">
         <v>3000</v>
@@ -2287,25 +2287,25 @@
         <v>3000</v>
       </c>
       <c r="X15" t="n">
-        <v>59.71739163763709</v>
+        <v>58.00000000000001</v>
       </c>
       <c r="Y15" t="n">
-        <v>4.558844833296899</v>
+        <v>6.340414684271129</v>
       </c>
       <c r="Z15" t="n">
-        <v>2.70646450620042</v>
+        <v>2.925925826310943</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.1130477991935698</v>
+        <v>0.108383693596484</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.03716841715414343</v>
+        <v>0.07492946116501936</v>
       </c>
       <c r="AC15" t="n">
         <v>58</v>
       </c>
       <c r="AD15" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE15" t="n">
         <v>0</v>
@@ -2334,59 +2334,59 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>45625.25</v>
+        <v>45624.54549155224</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>45625.75</v>
+        <v>45624.68828857363</v>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>12</v>
+        <v>3.427128513333333</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>period_2</t>
+          <t>preplan</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0108</t>
+          <t>WED01_LT01_3002</t>
         </is>
       </c>
       <c r="I16" t="n">
         <v>0.33</v>
       </c>
       <c r="J16" t="n">
-        <v>35345.61978727223</v>
+        <v>69950.69999999998</v>
       </c>
       <c r="K16" t="n">
-        <v>12000</v>
+        <v>3427.128513333334</v>
       </c>
       <c r="L16" t="n">
-        <v>23345.61978727223</v>
+        <v>66523.57148666665</v>
       </c>
       <c r="M16" t="n">
-        <v>58.27074099617414</v>
+        <v>55.15692796963216</v>
       </c>
       <c r="N16" t="n">
-        <v>4.542733948530114</v>
+        <v>9.041974529664218</v>
       </c>
       <c r="O16" t="n">
-        <v>3.182296227283953</v>
+        <v>3.905221911630801</v>
       </c>
       <c r="P16" t="n">
-        <v>0.1058319868276335</v>
+        <v>0.1058272675262239</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.03628485018586616</v>
+        <v>0.1531603422776934</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
@@ -2400,57 +2400,2131 @@
         <v>1000</v>
       </c>
       <c r="U16" t="n">
+        <v>10281.38554</v>
+      </c>
+      <c r="V16" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W16" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X16" t="n">
+        <v>58.00000000000001</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>6.340414684271129</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>2.925925826310943</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0.108383693596484</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>0.07492946116501936</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>45624.54549155224</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>45624.68828857363</v>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3.427128513333333</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>WES01_LT01_0901</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J17" t="n">
+        <v>22054.94778763339</v>
+      </c>
+      <c r="K17" t="n">
+        <v>56.84740245139484</v>
+      </c>
+      <c r="L17" t="n">
+        <v>21998.100385182</v>
+      </c>
+      <c r="M17" t="n">
+        <v>40.56124264065325</v>
+      </c>
+      <c r="N17" t="n">
+        <v>34.35151127901289</v>
+      </c>
+      <c r="O17" t="n">
+        <v>2.56585767038744</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0.1061514784064821</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.15325294075118</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T17" t="n">
+        <v>16.58747322437094</v>
+      </c>
+      <c r="U17" t="n">
+        <v>10281.38554</v>
+      </c>
+      <c r="V17" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W17" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X17" t="n">
+        <v>58.00000000000001</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>6.340414684271129</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>2.925925826310943</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0.108383693596484</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>0.07492946116501936</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>45624.68828857363</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="C18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.481074232777778</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ELW01_LT01_1002</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J18" t="n">
+        <v>169892.6</v>
+      </c>
+      <c r="K18" t="n">
+        <v>907.3802441580805</v>
+      </c>
+      <c r="L18" t="n">
+        <v>168985.2197558419</v>
+      </c>
+      <c r="M18" t="n">
+        <v>55.5151216882904</v>
+      </c>
+      <c r="N18" t="n">
+        <v>7.823278870512185</v>
+      </c>
+      <c r="O18" t="n">
+        <v>5.135935178262569</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0.1093451173600558</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.03282938903565423</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T18" t="n">
+        <v>612.6500779480004</v>
+      </c>
+      <c r="U18" t="n">
+        <v>4443.222698333333</v>
+      </c>
+      <c r="V18" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W18" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X18" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>5.48947206046786</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>3.615894622011488</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>0.1020511633607738</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>0.03756694009545923</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>45624.68828857363</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="C19" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.481074232777778</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>ELW01_RP01_0212</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="J19" t="n">
+        <v>224912.0816123666</v>
+      </c>
+      <c r="K19" t="n">
+        <v>573.6939886196971</v>
+      </c>
+      <c r="L19" t="n">
+        <v>224338.3876237469</v>
+      </c>
+      <c r="M19" t="n">
+        <v>60.52178373729767</v>
+      </c>
+      <c r="N19" t="n">
+        <v>4.059457898875317</v>
+      </c>
+      <c r="O19" t="n">
+        <v>3.033311423801729</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.1912254150327387</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.04966826077403921</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T19" t="n">
+        <v>387.3499220519994</v>
+      </c>
+      <c r="U19" t="n">
+        <v>4443.222698333333</v>
+      </c>
+      <c r="V19" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W19" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X19" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>5.48947206046786</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>3.615894622011488</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>0.1020511633607738</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>0.03756694009545923</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>45624.68828857363</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="C20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1.481074232777778</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ELW01_RP01_0807</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J20" t="n">
+        <v>9821.334889118063</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1481.074232777778</v>
+      </c>
+      <c r="L20" t="n">
+        <v>8340.260656340286</v>
+      </c>
+      <c r="M20" t="n">
+        <v>59.57843439126294</v>
+      </c>
+      <c r="N20" t="n">
+        <v>4.225669895284223</v>
+      </c>
+      <c r="O20" t="n">
+        <v>2.502769386280923</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.1068578171766122</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.03796622173938611</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S20" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T20" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U20" t="n">
+        <v>4443.222698333333</v>
+      </c>
+      <c r="V20" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W20" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X20" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>5.48947206046786</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>3.615894622011488</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>0.1020511633607738</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>0.03756694009545923</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>45624.68828857363</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1.481074232777778</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>FLY01_RP01_0104</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J21" t="n">
+        <v>9295.772860000001</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1481.074232777778</v>
+      </c>
+      <c r="L21" t="n">
+        <v>7814.698627222223</v>
+      </c>
+      <c r="M21" t="n">
+        <v>56.96711376602299</v>
+      </c>
+      <c r="N21" t="n">
+        <v>5.877383175588395</v>
+      </c>
+      <c r="O21" t="n">
+        <v>4.023430448886061</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0.0582342286245451</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.03538267385603032</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S21" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T21" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U21" t="n">
+        <v>4443.222698333333</v>
+      </c>
+      <c r="V21" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W21" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X21" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>5.48947206046786</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>3.615894622011488</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>0.1020511633607738</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>0.03756694009545923</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="C22" t="n">
+        <v>5</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>6</v>
+      </c>
+      <c r="F22" t="n">
+        <v>7.814698627222223</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>CEN01_RP01_0105</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J22" t="n">
+        <v>231608.4442305336</v>
+      </c>
+      <c r="K22" t="n">
+        <v>7814.698627222223</v>
+      </c>
+      <c r="L22" t="n">
+        <v>223793.7456033114</v>
+      </c>
+      <c r="M22" t="n">
+        <v>59.58008479807087</v>
+      </c>
+      <c r="N22" t="n">
+        <v>5.253888040550701</v>
+      </c>
+      <c r="O22" t="n">
+        <v>2.368739705797716</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0.1124777124620528</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.03174950411324488</v>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S22" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T22" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U22" t="n">
+        <v>23444.09588166667</v>
+      </c>
+      <c r="V22" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W22" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X22" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>6.01366437766795</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>3.308086888113809</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>0.1043616940809951</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>0.05866780113753148</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH22" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="C23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>6</v>
+      </c>
+      <c r="F23" t="n">
+        <v>7.814698627222223</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>ELW01_RP01_0212</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="J23" t="n">
+        <v>224338.3876237469</v>
+      </c>
+      <c r="K23" t="n">
+        <v>3344.27615618348</v>
+      </c>
+      <c r="L23" t="n">
+        <v>220994.1114675634</v>
+      </c>
+      <c r="M23" t="n">
+        <v>60.52178373729767</v>
+      </c>
+      <c r="N23" t="n">
+        <v>4.059457898875317</v>
+      </c>
+      <c r="O23" t="n">
+        <v>3.033311423801729</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.1912254150327387</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.04966826077403921</v>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S23" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T23" t="n">
+        <v>427.9469133376191</v>
+      </c>
+      <c r="U23" t="n">
+        <v>23444.09588166667</v>
+      </c>
+      <c r="V23" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W23" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X23" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>6.01366437766795</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>3.308086888113809</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>0.1043616940809951</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>0.05866780113753148</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH23" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL23" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="C24" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>6</v>
+      </c>
+      <c r="F24" t="n">
+        <v>7.814698627222223</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>FLY01_RP01_0104</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J24" t="n">
+        <v>7814.698627222223</v>
+      </c>
+      <c r="K24" t="n">
+        <v>7814.698627222223</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>56.96711376602299</v>
+      </c>
+      <c r="N24" t="n">
+        <v>5.877383175588395</v>
+      </c>
+      <c r="O24" t="n">
+        <v>4.023430448886061</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.0582342286245451</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.03538267385603032</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S24" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T24" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U24" t="n">
+        <v>23444.09588166667</v>
+      </c>
+      <c r="V24" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W24" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X24" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>6.01366437766795</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>3.308086888113809</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>0.1043616940809951</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>0.05866780113753148</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH24" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="C25" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>6</v>
+      </c>
+      <c r="F25" t="n">
+        <v>7.814698627222223</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>WED01_LT01_3002</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="J25" t="n">
+        <v>66523.57148666665</v>
+      </c>
+      <c r="K25" t="n">
+        <v>4470.422471038742</v>
+      </c>
+      <c r="L25" t="n">
+        <v>62053.14901562791</v>
+      </c>
+      <c r="M25" t="n">
+        <v>55.15692796963216</v>
+      </c>
+      <c r="N25" t="n">
+        <v>9.041974529664218</v>
+      </c>
+      <c r="O25" t="n">
+        <v>3.905221911630801</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0.1058272675262239</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0.1531603422776934</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T25" t="n">
+        <v>572.0530866623807</v>
+      </c>
+      <c r="U25" t="n">
+        <v>23444.09588166667</v>
+      </c>
+      <c r="V25" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W25" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X25" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>6.01366437766795</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>3.308086888113809</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>0.1043616940809951</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>0.05866780113753148</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="C26" t="n">
+        <v>6</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4.185301372777777</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>CEN01_RP01_0105</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J26" t="n">
+        <v>223793.7456033114</v>
+      </c>
+      <c r="K26" t="n">
+        <v>4185.301372777777</v>
+      </c>
+      <c r="L26" t="n">
+        <v>219608.4442305336</v>
+      </c>
+      <c r="M26" t="n">
+        <v>59.58008479807087</v>
+      </c>
+      <c r="N26" t="n">
+        <v>5.253888040550701</v>
+      </c>
+      <c r="O26" t="n">
+        <v>2.368739705797716</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0.1124777124620528</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0.03174950411324488</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S26" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T26" t="n">
+        <v>999.9999999999999</v>
+      </c>
+      <c r="U26" t="n">
+        <v>12555.90411833333</v>
+      </c>
+      <c r="V26" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W26" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X26" t="n">
+        <v>57.99999999999999</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="C27" t="n">
+        <v>6</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7</v>
+      </c>
+      <c r="F27" t="n">
+        <v>4.185301372777777</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>ELW01_LT01_3001</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J27" t="n">
+        <v>30246</v>
+      </c>
+      <c r="K27" t="n">
+        <v>651.1550548067353</v>
+      </c>
+      <c r="L27" t="n">
+        <v>29594.84494519327</v>
+      </c>
+      <c r="M27" t="n">
+        <v>52.43086483628262</v>
+      </c>
+      <c r="N27" t="n">
+        <v>10.3780597332974</v>
+      </c>
+      <c r="O27" t="n">
+        <v>4.752404239071938</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0.1197505789934543</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0.03023434519128211</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S27" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T27" t="n">
+        <v>155.5814018655877</v>
+      </c>
+      <c r="U27" t="n">
+        <v>12555.90411833333</v>
+      </c>
+      <c r="V27" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W27" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X27" t="n">
+        <v>57.99999999999999</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="C28" t="n">
+        <v>6</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>7</v>
+      </c>
+      <c r="F28" t="n">
+        <v>4.185301372777777</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>ELW01_RP01_0212</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J28" t="n">
+        <v>220994.1114675634</v>
+      </c>
+      <c r="K28" t="n">
+        <v>3534.146317971043</v>
+      </c>
+      <c r="L28" t="n">
+        <v>217459.9651495924</v>
+      </c>
+      <c r="M28" t="n">
+        <v>60.52178373729767</v>
+      </c>
+      <c r="N28" t="n">
+        <v>4.059457898875317</v>
+      </c>
+      <c r="O28" t="n">
+        <v>3.033311423801729</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0.1912254150327387</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0.04966826077403921</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S28" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T28" t="n">
+        <v>844.4185981344124</v>
+      </c>
+      <c r="U28" t="n">
+        <v>12555.90411833333</v>
+      </c>
+      <c r="V28" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W28" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X28" t="n">
+        <v>57.99999999999999</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB28" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ28" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="C29" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>7</v>
+      </c>
+      <c r="F29" t="n">
+        <v>4.185301372777777</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>WED01_LT01_3002</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J29" t="n">
+        <v>62053.14901562791</v>
+      </c>
+      <c r="K29" t="n">
+        <v>4185.301372777777</v>
+      </c>
+      <c r="L29" t="n">
+        <v>57867.84764285013</v>
+      </c>
+      <c r="M29" t="n">
+        <v>55.15692796963216</v>
+      </c>
+      <c r="N29" t="n">
+        <v>9.041974529664218</v>
+      </c>
+      <c r="O29" t="n">
+        <v>3.905221911630801</v>
+      </c>
+      <c r="P29" t="n">
+        <v>0.1058272675262239</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0.1531603422776934</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S29" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T29" t="n">
+        <v>999.9999999999999</v>
+      </c>
+      <c r="U29" t="n">
+        <v>12555.90411833333</v>
+      </c>
+      <c r="V29" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W29" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X29" t="n">
+        <v>57.99999999999999</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA29" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB29" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH29" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ29" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL29" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>45625.75</v>
+      </c>
+      <c r="C30" t="n">
+        <v>7</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>8</v>
+      </c>
+      <c r="F30" t="n">
+        <v>12</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>period_2</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>CEN01_RP01_0105</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J30" t="n">
+        <v>219608.4442305336</v>
+      </c>
+      <c r="K30" t="n">
+        <v>12000</v>
+      </c>
+      <c r="L30" t="n">
+        <v>207608.4442305336</v>
+      </c>
+      <c r="M30" t="n">
+        <v>59.58008479807087</v>
+      </c>
+      <c r="N30" t="n">
+        <v>5.253888040550701</v>
+      </c>
+      <c r="O30" t="n">
+        <v>2.368739705797716</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0.1124777124620528</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>0.03174950411324488</v>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S30" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T30" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U30" t="n">
         <v>36000</v>
       </c>
-      <c r="V16" t="n">
-        <v>3000</v>
-      </c>
-      <c r="W16" t="n">
-        <v>3000</v>
-      </c>
-      <c r="X16" t="n">
-        <v>59.71739163763709</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>4.558844833296899</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>2.70646450620042</v>
-      </c>
-      <c r="AA16" t="n">
-        <v>0.1130477991935698</v>
-      </c>
-      <c r="AB16" t="n">
-        <v>0.03716841715414343</v>
-      </c>
-      <c r="AC16" t="n">
-        <v>58</v>
-      </c>
-      <c r="AD16" t="n">
-        <v>61</v>
-      </c>
-      <c r="AE16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF16" t="n">
-        <v>100</v>
-      </c>
-      <c r="AG16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH16" t="n">
-        <v>100</v>
-      </c>
-      <c r="AI16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ16" t="n">
-        <v>100</v>
-      </c>
-      <c r="AK16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL16" t="n">
+      <c r="V30" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W30" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X30" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH30" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ30" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL30" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>45625.75</v>
+      </c>
+      <c r="C31" t="n">
+        <v>7</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>8</v>
+      </c>
+      <c r="F31" t="n">
+        <v>12</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>period_2</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>ELW01_LT01_3001</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J31" t="n">
+        <v>29594.84494519327</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1866.976822387052</v>
+      </c>
+      <c r="L31" t="n">
+        <v>27727.86812280622</v>
+      </c>
+      <c r="M31" t="n">
+        <v>52.43086483628262</v>
+      </c>
+      <c r="N31" t="n">
+        <v>10.3780597332974</v>
+      </c>
+      <c r="O31" t="n">
+        <v>4.752404239071938</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0.1197505789934543</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0.03023434519128211</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S31" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T31" t="n">
+        <v>155.5814018655877</v>
+      </c>
+      <c r="U31" t="n">
+        <v>36000</v>
+      </c>
+      <c r="V31" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W31" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X31" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH31" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>45625.75</v>
+      </c>
+      <c r="C32" t="n">
+        <v>7</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>8</v>
+      </c>
+      <c r="F32" t="n">
+        <v>12</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>period_2</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>ELW01_RP01_0212</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J32" t="n">
+        <v>217459.9651495924</v>
+      </c>
+      <c r="K32" t="n">
+        <v>10133.02317761295</v>
+      </c>
+      <c r="L32" t="n">
+        <v>207326.9419719794</v>
+      </c>
+      <c r="M32" t="n">
+        <v>60.52178373729767</v>
+      </c>
+      <c r="N32" t="n">
+        <v>4.059457898875317</v>
+      </c>
+      <c r="O32" t="n">
+        <v>3.033311423801729</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0.1912254150327387</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0.04966826077403921</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S32" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T32" t="n">
+        <v>844.4185981344123</v>
+      </c>
+      <c r="U32" t="n">
+        <v>36000</v>
+      </c>
+      <c r="V32" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W32" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X32" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB32" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH32" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ32" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>45625.75</v>
+      </c>
+      <c r="C33" t="n">
+        <v>7</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>8</v>
+      </c>
+      <c r="F33" t="n">
+        <v>12</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>period_2</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>WED01_LT01_3002</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J33" t="n">
+        <v>57867.84764285013</v>
+      </c>
+      <c r="K33" t="n">
+        <v>12000</v>
+      </c>
+      <c r="L33" t="n">
+        <v>45867.84764285013</v>
+      </c>
+      <c r="M33" t="n">
+        <v>55.15692796963216</v>
+      </c>
+      <c r="N33" t="n">
+        <v>9.041974529664218</v>
+      </c>
+      <c r="O33" t="n">
+        <v>3.905221911630801</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0.1058272675262239</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0.1531603422776934</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S33" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T33" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U33" t="n">
+        <v>36000</v>
+      </c>
+      <c r="V33" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W33" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X33" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB33" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH33" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ33" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL33" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Gantt chart and table of blend details implemented in the main GUI.
Next:
1. CaseModeller user interactions (blend mode 2)
2. Implement stockpile profiles in the GUI
3. Start Blending Dashboard (manual Gantt)
</commit_message>
<xml_diff>
--- a/blendmaster_OOP/output/optimised_blend_report_2024-11-28_06-00.xlsx
+++ b/blendmaster_OOP/output/optimised_blend_report_2024-11-28_06-00.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL6"/>
+  <dimension ref="A1:AL33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,7 +629,7 @@
         <v>45624.25</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45624.54549155224</v>
+        <v>45624.26702842084</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -638,10 +638,10 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>7.091797253888889</v>
+        <v>0.4086820999999999</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -650,35 +650,35 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CEN01_LT01_1001</t>
+          <t>ELW01_RP01_0212</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>0.26</v>
       </c>
       <c r="J2" t="n">
-        <v>37152.89999999999</v>
+        <v>225234.6115</v>
       </c>
       <c r="K2" t="n">
-        <v>7091.797253888889</v>
+        <v>322.5298876333841</v>
       </c>
       <c r="L2" t="n">
-        <v>30061.1027461111</v>
+        <v>224912.0816123666</v>
       </c>
       <c r="M2" t="n">
-        <v>54.45474593268222</v>
+        <v>60.52178373729767</v>
       </c>
       <c r="N2" t="n">
-        <v>8.521316771514254</v>
+        <v>4.059457898875317</v>
       </c>
       <c r="O2" t="n">
-        <v>5.719285475110874</v>
+        <v>3.033311423801729</v>
       </c>
       <c r="P2" t="n">
-        <v>0.1656054369029566</v>
+        <v>0.1912254150327387</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.05286775893613377</v>
+        <v>0.04966826077403921</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -689,37 +689,37 @@
         <v>1000</v>
       </c>
       <c r="T2" t="n">
-        <v>1000</v>
+        <v>789.1950433683886</v>
       </c>
       <c r="U2" t="n">
-        <v>7091.797253888889</v>
+        <v>1226.0463</v>
       </c>
       <c r="V2" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="W2" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="X2" t="n">
-        <v>54.45474593268222</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="Y2" t="n">
-        <v>8.521316771514254</v>
+        <v>6.098594256090682</v>
       </c>
       <c r="Z2" t="n">
-        <v>5.719285475110874</v>
+        <v>3.868554741238664</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.1656054369029566</v>
+        <v>0.1145784485168504</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.05286775893613377</v>
+        <v>0.04956257802280711</v>
       </c>
       <c r="AC2" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="AD2" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
@@ -748,22 +748,22 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45624.54549155224</v>
+        <v>45624.25</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45624.68828857363</v>
+        <v>45624.26702842084</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>3.427128513333333</v>
+        <v>0.4086820999999999</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -772,35 +772,35 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>CEN01_LT01_1001</t>
+          <t>FLY01_RP01_0801</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0.33</v>
       </c>
       <c r="J3" t="n">
-        <v>30061.1027461111</v>
+        <v>408.6820999999999</v>
       </c>
       <c r="K3" t="n">
-        <v>3427.128513333334</v>
+        <v>408.6820999999999</v>
       </c>
       <c r="L3" t="n">
-        <v>26633.97423277777</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>54.45474593268222</v>
+        <v>55.56862076349383</v>
       </c>
       <c r="N3" t="n">
-        <v>8.521316771514254</v>
+        <v>4.715978440440851</v>
       </c>
       <c r="O3" t="n">
-        <v>5.719285475110874</v>
+        <v>5.580065987524456</v>
       </c>
       <c r="P3" t="n">
-        <v>0.1656054369029566</v>
+        <v>0.05066384624236227</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.05286775893613377</v>
+        <v>0.02174606032201762</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -814,34 +814,34 @@
         <v>1000</v>
       </c>
       <c r="U3" t="n">
-        <v>3427.128513333334</v>
+        <v>1226.0463</v>
       </c>
       <c r="V3" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="W3" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="X3" t="n">
-        <v>54.45474593268222</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="Y3" t="n">
-        <v>8.521316771514254</v>
+        <v>6.098594256090682</v>
       </c>
       <c r="Z3" t="n">
-        <v>5.719285475110874</v>
+        <v>3.868554741238664</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.1656054369029566</v>
+        <v>0.1145784485168504</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.05286775893613377</v>
+        <v>0.04956257802280711</v>
       </c>
       <c r="AC3" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="AD3" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="AE3" t="n">
         <v>0</v>
@@ -870,22 +870,22 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45624.68828857363</v>
+        <v>45624.25</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45624.75</v>
+        <v>45624.26702842084</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>1.481074232777778</v>
+        <v>0.4086820999999999</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -894,35 +894,35 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CEN01_LT01_1001</t>
+          <t>WED01_RP01_0703</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0.33</v>
       </c>
       <c r="J4" t="n">
-        <v>26633.97423277777</v>
+        <v>1813.5</v>
       </c>
       <c r="K4" t="n">
-        <v>1481.074232777778</v>
+        <v>408.6820999999999</v>
       </c>
       <c r="L4" t="n">
-        <v>25152.89999999999</v>
+        <v>1404.8179</v>
       </c>
       <c r="M4" t="n">
-        <v>54.45474593268222</v>
+        <v>62.11737649943012</v>
       </c>
       <c r="N4" t="n">
-        <v>8.521316771514254</v>
+        <v>3.134631429873529</v>
       </c>
       <c r="O4" t="n">
-        <v>5.719285475110874</v>
+        <v>3.090828380605592</v>
       </c>
       <c r="P4" t="n">
-        <v>0.1656054369029566</v>
+        <v>0.1197800917964288</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.05286775893613377</v>
+        <v>0.05543724900208404</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -936,34 +936,34 @@
         <v>1000</v>
       </c>
       <c r="U4" t="n">
-        <v>1481.074232777778</v>
+        <v>1226.0463</v>
       </c>
       <c r="V4" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="W4" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="X4" t="n">
-        <v>54.45474593268222</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="Y4" t="n">
-        <v>8.521316771514254</v>
+        <v>6.098594256090682</v>
       </c>
       <c r="Z4" t="n">
-        <v>5.719285475110874</v>
+        <v>3.868554741238664</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.1656054369029566</v>
+        <v>0.1145784485168504</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.05286775893613377</v>
+        <v>0.04956257802280711</v>
       </c>
       <c r="AC4" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="AD4" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
@@ -992,59 +992,59 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45624.75</v>
+        <v>45624.25</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45625.25</v>
+        <v>45624.26702842084</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>12</v>
+        <v>0.4086820999999999</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>period_1</t>
+          <t>preplan</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CEN01_LT01_1001</t>
+          <t>WES01_LT01_0901</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>25152.89999999999</v>
+        <v>22141.10000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>12000</v>
+        <v>86.1522123666158</v>
       </c>
       <c r="L5" t="n">
-        <v>13152.89999999999</v>
+        <v>22054.94778763339</v>
       </c>
       <c r="M5" t="n">
-        <v>54.45474593268222</v>
+        <v>40.56124264065325</v>
       </c>
       <c r="N5" t="n">
-        <v>8.521316771514254</v>
+        <v>34.35151127901289</v>
       </c>
       <c r="O5" t="n">
-        <v>5.719285475110874</v>
+        <v>2.56585767038744</v>
       </c>
       <c r="P5" t="n">
-        <v>0.1656054369029566</v>
+        <v>0.1061514784064821</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.05286775893613377</v>
+        <v>0.15325294075118</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -1055,37 +1055,37 @@
         <v>1000</v>
       </c>
       <c r="T5" t="n">
-        <v>1000</v>
+        <v>210.8049566316112</v>
       </c>
       <c r="U5" t="n">
-        <v>12000</v>
+        <v>1226.0463</v>
       </c>
       <c r="V5" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="W5" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="X5" t="n">
-        <v>54.45474593268222</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="Y5" t="n">
-        <v>8.521316771514254</v>
+        <v>6.098594256090682</v>
       </c>
       <c r="Z5" t="n">
-        <v>5.719285475110874</v>
+        <v>3.868554741238664</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.1656054369029566</v>
+        <v>0.1145784485168504</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.05286775893613378</v>
+        <v>0.04956257802280711</v>
       </c>
       <c r="AC5" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="AD5" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
@@ -1114,13 +1114,13 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45625.25</v>
+        <v>45624.26702842084</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45625.75</v>
+        <v>45624.3255625</v>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
@@ -1129,44 +1129,44 @@
         <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>12</v>
+        <v>1.4048179</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>period_2</t>
+          <t>preplan</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CEN01_LT01_1001</t>
+          <t>CEN01_RP01_0109</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0.03</v>
       </c>
       <c r="J6" t="n">
-        <v>13152.89999999999</v>
+        <v>363724.09875</v>
       </c>
       <c r="K6" t="n">
-        <v>12000</v>
+        <v>143.66747301729</v>
       </c>
       <c r="L6" t="n">
-        <v>1152.899999999994</v>
+        <v>363580.4312769827</v>
       </c>
       <c r="M6" t="n">
-        <v>54.45474593268222</v>
+        <v>61.79549201427914</v>
       </c>
       <c r="N6" t="n">
-        <v>8.521316771514254</v>
+        <v>3.909353754397719</v>
       </c>
       <c r="O6" t="n">
-        <v>5.719285475110874</v>
+        <v>2.306220477075012</v>
       </c>
       <c r="P6" t="n">
-        <v>0.1656054369029566</v>
+        <v>0.1221413849964776</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.05286775893613377</v>
+        <v>0.03605561216887876</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1177,60 +1177,3354 @@
         <v>1000</v>
       </c>
       <c r="T6" t="n">
+        <v>102.2676839591024</v>
+      </c>
+      <c r="U6" t="n">
+        <v>4214.4537</v>
+      </c>
+      <c r="V6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X6" t="n">
+        <v>58.00000000000001</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>6.019595554336112</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>4.115528309395112</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0.1166994619512664</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0.04877589831351777</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>45624.26702842084</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>45624.3255625</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.4048179</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ELW01_LT01_2001</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1048985.1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1404.8179</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1047580.2821</v>
+      </c>
+      <c r="M7" t="n">
+        <v>56.26801388728946</v>
+      </c>
+      <c r="N7" t="n">
+        <v>6.935902734745083</v>
+      </c>
+      <c r="O7" t="n">
+        <v>4.976544911650335</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.1237568390236727</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.05754207494577221</v>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S7" t="n">
         <v>1000</v>
       </c>
-      <c r="U6" t="n">
+      <c r="T7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U7" t="n">
+        <v>4214.4537</v>
+      </c>
+      <c r="V7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X7" t="n">
+        <v>58.00000000000001</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>6.019595554336112</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>4.115528309395112</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>0.1166994619512664</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0.04877589831351777</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>45624.26702842084</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>45624.3255625</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.4048179</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>WED01_RP01_0703</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1404.8179</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1404.8179</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>62.11737649943012</v>
+      </c>
+      <c r="N8" t="n">
+        <v>3.134631429873529</v>
+      </c>
+      <c r="O8" t="n">
+        <v>3.090828380605592</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.1197800917964288</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.05543724900208404</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U8" t="n">
+        <v>4214.4537</v>
+      </c>
+      <c r="V8" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W8" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X8" t="n">
+        <v>58.00000000000001</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>6.019595554336112</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>4.115528309395112</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>0.1166994619512664</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>0.04877589831351777</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>45624.26702842084</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>45624.3255625</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.4048179</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>WES01_LT01_2001</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J9" t="n">
+        <v>714322.3000000004</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1261.15042698271</v>
+      </c>
+      <c r="L9" t="n">
+        <v>713061.1495730177</v>
+      </c>
+      <c r="M9" t="n">
+        <v>54.91049713266775</v>
+      </c>
+      <c r="N9" t="n">
+        <v>8.452911640316779</v>
+      </c>
+      <c r="O9" t="n">
+        <v>4.503970433939116</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.1047866238005244</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.03303996805335782</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T9" t="n">
+        <v>897.7323160408976</v>
+      </c>
+      <c r="U9" t="n">
+        <v>4214.4537</v>
+      </c>
+      <c r="V9" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W9" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X9" t="n">
+        <v>58.00000000000001</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>6.019595554336112</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>4.115528309395112</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>0.1166994619512664</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>0.04877589831351777</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>45624.3255625</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>45624.54549155224</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5.278297253888889</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>CEN01_RP01_0105</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J10" t="n">
+        <v>236195.31475</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1159.742006133012</v>
+      </c>
+      <c r="L10" t="n">
+        <v>235035.5727438669</v>
+      </c>
+      <c r="M10" t="n">
+        <v>59.58008479807087</v>
+      </c>
+      <c r="N10" t="n">
+        <v>5.253888040550701</v>
+      </c>
+      <c r="O10" t="n">
+        <v>2.368739705797716</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.1124777124620528</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.03174950411324488</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T10" t="n">
+        <v>219.7189643456608</v>
+      </c>
+      <c r="U10" t="n">
+        <v>15834.89176166667</v>
+      </c>
+      <c r="V10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X10" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>6.198427325733884</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>3.772528379479401</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0.1174582419520254</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>0.04211803858918725</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>45624.3255625</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>45624.54549155224</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5.278297253888889</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>CEN01_RP01_0109</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J11" t="n">
+        <v>363580.4312769827</v>
+      </c>
+      <c r="K11" t="n">
+        <v>5278.297253888889</v>
+      </c>
+      <c r="L11" t="n">
+        <v>358302.1340230938</v>
+      </c>
+      <c r="M11" t="n">
+        <v>61.79549201427914</v>
+      </c>
+      <c r="N11" t="n">
+        <v>3.909353754397719</v>
+      </c>
+      <c r="O11" t="n">
+        <v>2.306220477075012</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.1221413849964776</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.03605561216887876</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U11" t="n">
+        <v>15834.89176166667</v>
+      </c>
+      <c r="V11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X11" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>6.198427325733884</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>3.772528379479401</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0.1174582419520254</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>0.04211803858918725</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>45624.3255625</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>45624.54549155224</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5.278297253888889</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>ELW01_LT01_2001</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1047580.2821</v>
+      </c>
+      <c r="K12" t="n">
+        <v>5278.297253888889</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1042301.984846111</v>
+      </c>
+      <c r="M12" t="n">
+        <v>56.26801388728946</v>
+      </c>
+      <c r="N12" t="n">
+        <v>6.935902734745083</v>
+      </c>
+      <c r="O12" t="n">
+        <v>4.976544911650335</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.1237568390236727</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.05754207494577221</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U12" t="n">
+        <v>15834.89176166667</v>
+      </c>
+      <c r="V12" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W12" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X12" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>6.198427325733884</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>3.772528379479401</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>0.1174582419520254</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>0.04211803858918725</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>45624.3255625</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>45624.54549155224</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" t="n">
+        <v>5.278297253888889</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>WES01_LT01_2001</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="J13" t="n">
+        <v>713061.1495730177</v>
+      </c>
+      <c r="K13" t="n">
+        <v>4118.555247755876</v>
+      </c>
+      <c r="L13" t="n">
+        <v>708942.5943252619</v>
+      </c>
+      <c r="M13" t="n">
+        <v>54.91049713266775</v>
+      </c>
+      <c r="N13" t="n">
+        <v>8.452911640316779</v>
+      </c>
+      <c r="O13" t="n">
+        <v>4.503970433939116</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.1047866238005244</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.03303996805335782</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S13" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T13" t="n">
+        <v>780.281035654339</v>
+      </c>
+      <c r="U13" t="n">
+        <v>15834.89176166667</v>
+      </c>
+      <c r="V13" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W13" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X13" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>6.198427325733884</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>3.772528379479401</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>0.1174582419520254</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>0.04211803858918725</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>45624.54549155224</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>45624.68828857363</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" t="n">
+        <v>3.427128513333333</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>CEN01_RP01_0105</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J14" t="n">
+        <v>235035.5727438669</v>
+      </c>
+      <c r="K14" t="n">
+        <v>3427.128513333334</v>
+      </c>
+      <c r="L14" t="n">
+        <v>231608.4442305336</v>
+      </c>
+      <c r="M14" t="n">
+        <v>59.58008479807087</v>
+      </c>
+      <c r="N14" t="n">
+        <v>5.253888040550701</v>
+      </c>
+      <c r="O14" t="n">
+        <v>2.368739705797716</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.1124777124620528</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0.03174950411324488</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U14" t="n">
+        <v>10281.38554</v>
+      </c>
+      <c r="V14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X14" t="n">
+        <v>58.00000000000001</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>6.340414684271129</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>2.925925826310943</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>0.108383693596484</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>0.07492946116501936</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>45624.54549155224</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>45624.68828857363</v>
+      </c>
+      <c r="C15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3.427128513333333</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>ELW01_RP01_0807</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J15" t="n">
+        <v>13191.616</v>
+      </c>
+      <c r="K15" t="n">
+        <v>3370.281110881937</v>
+      </c>
+      <c r="L15" t="n">
+        <v>9821.334889118063</v>
+      </c>
+      <c r="M15" t="n">
+        <v>59.57843439126294</v>
+      </c>
+      <c r="N15" t="n">
+        <v>4.225669895284223</v>
+      </c>
+      <c r="O15" t="n">
+        <v>2.502769386280923</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0.1068578171766122</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.03796622173938611</v>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T15" t="n">
+        <v>983.4125267756287</v>
+      </c>
+      <c r="U15" t="n">
+        <v>10281.38554</v>
+      </c>
+      <c r="V15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X15" t="n">
+        <v>58.00000000000001</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>6.340414684271129</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>2.925925826310943</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0.108383693596484</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>0.07492946116501936</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>45624.54549155224</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>45624.68828857363</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" t="n">
+        <v>3.427128513333333</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>WED01_LT01_3002</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J16" t="n">
+        <v>69950.69999999998</v>
+      </c>
+      <c r="K16" t="n">
+        <v>3427.128513333334</v>
+      </c>
+      <c r="L16" t="n">
+        <v>66523.57148666665</v>
+      </c>
+      <c r="M16" t="n">
+        <v>55.15692796963216</v>
+      </c>
+      <c r="N16" t="n">
+        <v>9.041974529664218</v>
+      </c>
+      <c r="O16" t="n">
+        <v>3.905221911630801</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0.1058272675262239</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0.1531603422776934</v>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S16" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T16" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U16" t="n">
+        <v>10281.38554</v>
+      </c>
+      <c r="V16" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W16" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X16" t="n">
+        <v>58.00000000000001</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>6.340414684271129</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>2.925925826310943</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0.108383693596484</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>0.07492946116501936</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>45624.54549155224</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>45624.68828857363</v>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3.427128513333333</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>WES01_LT01_0901</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J17" t="n">
+        <v>22054.94778763339</v>
+      </c>
+      <c r="K17" t="n">
+        <v>56.84740245139484</v>
+      </c>
+      <c r="L17" t="n">
+        <v>21998.100385182</v>
+      </c>
+      <c r="M17" t="n">
+        <v>40.56124264065325</v>
+      </c>
+      <c r="N17" t="n">
+        <v>34.35151127901289</v>
+      </c>
+      <c r="O17" t="n">
+        <v>2.56585767038744</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0.1061514784064821</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.15325294075118</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T17" t="n">
+        <v>16.58747322437094</v>
+      </c>
+      <c r="U17" t="n">
+        <v>10281.38554</v>
+      </c>
+      <c r="V17" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W17" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X17" t="n">
+        <v>58.00000000000001</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>6.340414684271129</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>2.925925826310943</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0.108383693596484</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>0.07492946116501936</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>45624.68828857363</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="C18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.481074232777778</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ELW01_LT01_1002</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J18" t="n">
+        <v>169892.6</v>
+      </c>
+      <c r="K18" t="n">
+        <v>907.3802441580805</v>
+      </c>
+      <c r="L18" t="n">
+        <v>168985.2197558419</v>
+      </c>
+      <c r="M18" t="n">
+        <v>55.5151216882904</v>
+      </c>
+      <c r="N18" t="n">
+        <v>7.823278870512185</v>
+      </c>
+      <c r="O18" t="n">
+        <v>5.135935178262569</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0.1093451173600558</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.03282938903565423</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T18" t="n">
+        <v>612.6500779480004</v>
+      </c>
+      <c r="U18" t="n">
+        <v>4443.222698333333</v>
+      </c>
+      <c r="V18" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W18" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X18" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>5.48947206046786</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>3.615894622011488</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>0.1020511633607738</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>0.03756694009545923</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>45624.68828857363</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="C19" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.481074232777778</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>ELW01_RP01_0212</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="J19" t="n">
+        <v>224912.0816123666</v>
+      </c>
+      <c r="K19" t="n">
+        <v>573.6939886196971</v>
+      </c>
+      <c r="L19" t="n">
+        <v>224338.3876237469</v>
+      </c>
+      <c r="M19" t="n">
+        <v>60.52178373729767</v>
+      </c>
+      <c r="N19" t="n">
+        <v>4.059457898875317</v>
+      </c>
+      <c r="O19" t="n">
+        <v>3.033311423801729</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.1912254150327387</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.04966826077403921</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T19" t="n">
+        <v>387.3499220519994</v>
+      </c>
+      <c r="U19" t="n">
+        <v>4443.222698333333</v>
+      </c>
+      <c r="V19" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W19" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X19" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>5.48947206046786</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>3.615894622011488</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>0.1020511633607738</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>0.03756694009545923</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>45624.68828857363</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="C20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1.481074232777778</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ELW01_RP01_0807</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J20" t="n">
+        <v>9821.334889118063</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1481.074232777778</v>
+      </c>
+      <c r="L20" t="n">
+        <v>8340.260656340286</v>
+      </c>
+      <c r="M20" t="n">
+        <v>59.57843439126294</v>
+      </c>
+      <c r="N20" t="n">
+        <v>4.225669895284223</v>
+      </c>
+      <c r="O20" t="n">
+        <v>2.502769386280923</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.1068578171766122</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.03796622173938611</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S20" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T20" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U20" t="n">
+        <v>4443.222698333333</v>
+      </c>
+      <c r="V20" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W20" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X20" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>5.48947206046786</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>3.615894622011488</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>0.1020511633607738</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>0.03756694009545923</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>45624.68828857363</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1.481074232777778</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>preplan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>FLY01_RP01_0104</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J21" t="n">
+        <v>9295.772860000001</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1481.074232777778</v>
+      </c>
+      <c r="L21" t="n">
+        <v>7814.698627222223</v>
+      </c>
+      <c r="M21" t="n">
+        <v>56.96711376602299</v>
+      </c>
+      <c r="N21" t="n">
+        <v>5.877383175588395</v>
+      </c>
+      <c r="O21" t="n">
+        <v>4.023430448886061</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0.0582342286245451</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.03538267385603032</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S21" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T21" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U21" t="n">
+        <v>4443.222698333333</v>
+      </c>
+      <c r="V21" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W21" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X21" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>5.48947206046786</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>3.615894622011488</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>0.1020511633607738</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>0.03756694009545923</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="C22" t="n">
+        <v>5</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>6</v>
+      </c>
+      <c r="F22" t="n">
+        <v>7.814698627222223</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>CEN01_RP01_0105</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J22" t="n">
+        <v>231608.4442305336</v>
+      </c>
+      <c r="K22" t="n">
+        <v>7814.698627222223</v>
+      </c>
+      <c r="L22" t="n">
+        <v>223793.7456033114</v>
+      </c>
+      <c r="M22" t="n">
+        <v>59.58008479807087</v>
+      </c>
+      <c r="N22" t="n">
+        <v>5.253888040550701</v>
+      </c>
+      <c r="O22" t="n">
+        <v>2.368739705797716</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0.1124777124620528</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.03174950411324488</v>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S22" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T22" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U22" t="n">
+        <v>23444.09588166667</v>
+      </c>
+      <c r="V22" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W22" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X22" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>6.01366437766795</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>3.308086888113809</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>0.1043616940809951</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>0.05866780113753148</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH22" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="C23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>6</v>
+      </c>
+      <c r="F23" t="n">
+        <v>7.814698627222223</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>ELW01_RP01_0212</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="J23" t="n">
+        <v>224338.3876237469</v>
+      </c>
+      <c r="K23" t="n">
+        <v>3344.27615618348</v>
+      </c>
+      <c r="L23" t="n">
+        <v>220994.1114675634</v>
+      </c>
+      <c r="M23" t="n">
+        <v>60.52178373729767</v>
+      </c>
+      <c r="N23" t="n">
+        <v>4.059457898875317</v>
+      </c>
+      <c r="O23" t="n">
+        <v>3.033311423801729</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.1912254150327387</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.04966826077403921</v>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S23" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T23" t="n">
+        <v>427.9469133376191</v>
+      </c>
+      <c r="U23" t="n">
+        <v>23444.09588166667</v>
+      </c>
+      <c r="V23" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W23" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X23" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>6.01366437766795</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>3.308086888113809</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>0.1043616940809951</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>0.05866780113753148</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH23" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL23" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="C24" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>6</v>
+      </c>
+      <c r="F24" t="n">
+        <v>7.814698627222223</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>FLY01_RP01_0104</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J24" t="n">
+        <v>7814.698627222223</v>
+      </c>
+      <c r="K24" t="n">
+        <v>7814.698627222223</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>56.96711376602299</v>
+      </c>
+      <c r="N24" t="n">
+        <v>5.877383175588395</v>
+      </c>
+      <c r="O24" t="n">
+        <v>4.023430448886061</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.0582342286245451</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.03538267385603032</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S24" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T24" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U24" t="n">
+        <v>23444.09588166667</v>
+      </c>
+      <c r="V24" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W24" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X24" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>6.01366437766795</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>3.308086888113809</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>0.1043616940809951</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>0.05866780113753148</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH24" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>45624.75</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="C25" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>6</v>
+      </c>
+      <c r="F25" t="n">
+        <v>7.814698627222223</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>WED01_LT01_3002</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="J25" t="n">
+        <v>66523.57148666665</v>
+      </c>
+      <c r="K25" t="n">
+        <v>4470.422471038742</v>
+      </c>
+      <c r="L25" t="n">
+        <v>62053.14901562791</v>
+      </c>
+      <c r="M25" t="n">
+        <v>55.15692796963216</v>
+      </c>
+      <c r="N25" t="n">
+        <v>9.041974529664218</v>
+      </c>
+      <c r="O25" t="n">
+        <v>3.905221911630801</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0.1058272675262239</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0.1531603422776934</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T25" t="n">
+        <v>572.0530866623807</v>
+      </c>
+      <c r="U25" t="n">
+        <v>23444.09588166667</v>
+      </c>
+      <c r="V25" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W25" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X25" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>6.01366437766795</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>3.308086888113809</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>0.1043616940809951</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>0.05866780113753148</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="C26" t="n">
+        <v>6</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4.185301372777777</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>CEN01_RP01_0105</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J26" t="n">
+        <v>223793.7456033114</v>
+      </c>
+      <c r="K26" t="n">
+        <v>4185.301372777777</v>
+      </c>
+      <c r="L26" t="n">
+        <v>219608.4442305336</v>
+      </c>
+      <c r="M26" t="n">
+        <v>59.58008479807087</v>
+      </c>
+      <c r="N26" t="n">
+        <v>5.253888040550701</v>
+      </c>
+      <c r="O26" t="n">
+        <v>2.368739705797716</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0.1124777124620528</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0.03174950411324488</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S26" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T26" t="n">
+        <v>999.9999999999999</v>
+      </c>
+      <c r="U26" t="n">
+        <v>12555.90411833333</v>
+      </c>
+      <c r="V26" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W26" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X26" t="n">
+        <v>57.99999999999999</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="C27" t="n">
+        <v>6</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7</v>
+      </c>
+      <c r="F27" t="n">
+        <v>4.185301372777777</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>ELW01_LT01_3001</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J27" t="n">
+        <v>30246</v>
+      </c>
+      <c r="K27" t="n">
+        <v>651.1550548067353</v>
+      </c>
+      <c r="L27" t="n">
+        <v>29594.84494519327</v>
+      </c>
+      <c r="M27" t="n">
+        <v>52.43086483628262</v>
+      </c>
+      <c r="N27" t="n">
+        <v>10.3780597332974</v>
+      </c>
+      <c r="O27" t="n">
+        <v>4.752404239071938</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0.1197505789934543</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0.03023434519128211</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S27" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T27" t="n">
+        <v>155.5814018655877</v>
+      </c>
+      <c r="U27" t="n">
+        <v>12555.90411833333</v>
+      </c>
+      <c r="V27" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W27" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X27" t="n">
+        <v>57.99999999999999</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="C28" t="n">
+        <v>6</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>7</v>
+      </c>
+      <c r="F28" t="n">
+        <v>4.185301372777777</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>ELW01_RP01_0212</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J28" t="n">
+        <v>220994.1114675634</v>
+      </c>
+      <c r="K28" t="n">
+        <v>3534.146317971043</v>
+      </c>
+      <c r="L28" t="n">
+        <v>217459.9651495924</v>
+      </c>
+      <c r="M28" t="n">
+        <v>60.52178373729767</v>
+      </c>
+      <c r="N28" t="n">
+        <v>4.059457898875317</v>
+      </c>
+      <c r="O28" t="n">
+        <v>3.033311423801729</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0.1912254150327387</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0.04966826077403921</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S28" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T28" t="n">
+        <v>844.4185981344124</v>
+      </c>
+      <c r="U28" t="n">
+        <v>12555.90411833333</v>
+      </c>
+      <c r="V28" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W28" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X28" t="n">
+        <v>57.99999999999999</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB28" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ28" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>45625.0756124428</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="C29" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>7</v>
+      </c>
+      <c r="F29" t="n">
+        <v>4.185301372777777</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>period_1</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>WED01_LT01_3002</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J29" t="n">
+        <v>62053.14901562791</v>
+      </c>
+      <c r="K29" t="n">
+        <v>4185.301372777777</v>
+      </c>
+      <c r="L29" t="n">
+        <v>57867.84764285013</v>
+      </c>
+      <c r="M29" t="n">
+        <v>55.15692796963216</v>
+      </c>
+      <c r="N29" t="n">
+        <v>9.041974529664218</v>
+      </c>
+      <c r="O29" t="n">
+        <v>3.905221911630801</v>
+      </c>
+      <c r="P29" t="n">
+        <v>0.1058272675262239</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0.1531603422776934</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S29" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T29" t="n">
+        <v>999.9999999999999</v>
+      </c>
+      <c r="U29" t="n">
+        <v>12555.90411833333</v>
+      </c>
+      <c r="V29" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W29" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X29" t="n">
+        <v>57.99999999999999</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA29" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB29" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH29" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ29" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL29" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>45625.75</v>
+      </c>
+      <c r="C30" t="n">
+        <v>7</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>8</v>
+      </c>
+      <c r="F30" t="n">
+        <v>12</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>period_2</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>CEN01_RP01_0105</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J30" t="n">
+        <v>219608.4442305336</v>
+      </c>
+      <c r="K30" t="n">
         <v>12000</v>
       </c>
-      <c r="V6" t="n">
+      <c r="L30" t="n">
+        <v>207608.4442305336</v>
+      </c>
+      <c r="M30" t="n">
+        <v>59.58008479807087</v>
+      </c>
+      <c r="N30" t="n">
+        <v>5.253888040550701</v>
+      </c>
+      <c r="O30" t="n">
+        <v>2.368739705797716</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0.1124777124620528</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>0.03174950411324488</v>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S30" t="n">
         <v>1000</v>
       </c>
-      <c r="W6" t="n">
+      <c r="T30" t="n">
         <v>1000</v>
       </c>
-      <c r="X6" t="n">
-        <v>54.45474593268222</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>8.521316771514254</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>5.719285475110874</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>0.1656054369029566</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>0.05286775893613378</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>100</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>100</v>
-      </c>
-      <c r="AG6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>100</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>100</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL6" t="n">
+      <c r="U30" t="n">
+        <v>36000</v>
+      </c>
+      <c r="V30" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W30" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X30" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH30" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ30" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL30" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>45625.75</v>
+      </c>
+      <c r="C31" t="n">
+        <v>7</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>8</v>
+      </c>
+      <c r="F31" t="n">
+        <v>12</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>period_2</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>ELW01_LT01_3001</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J31" t="n">
+        <v>29594.84494519327</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1866.976822387052</v>
+      </c>
+      <c r="L31" t="n">
+        <v>27727.86812280622</v>
+      </c>
+      <c r="M31" t="n">
+        <v>52.43086483628262</v>
+      </c>
+      <c r="N31" t="n">
+        <v>10.3780597332974</v>
+      </c>
+      <c r="O31" t="n">
+        <v>4.752404239071938</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0.1197505789934543</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0.03023434519128211</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S31" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T31" t="n">
+        <v>155.5814018655877</v>
+      </c>
+      <c r="U31" t="n">
+        <v>36000</v>
+      </c>
+      <c r="V31" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W31" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X31" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH31" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>45625.75</v>
+      </c>
+      <c r="C32" t="n">
+        <v>7</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>8</v>
+      </c>
+      <c r="F32" t="n">
+        <v>12</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>period_2</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>ELW01_RP01_0212</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J32" t="n">
+        <v>217459.9651495924</v>
+      </c>
+      <c r="K32" t="n">
+        <v>10133.02317761295</v>
+      </c>
+      <c r="L32" t="n">
+        <v>207326.9419719794</v>
+      </c>
+      <c r="M32" t="n">
+        <v>60.52178373729767</v>
+      </c>
+      <c r="N32" t="n">
+        <v>4.059457898875317</v>
+      </c>
+      <c r="O32" t="n">
+        <v>3.033311423801729</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0.1912254150327387</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0.04966826077403921</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S32" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T32" t="n">
+        <v>844.4185981344123</v>
+      </c>
+      <c r="U32" t="n">
+        <v>36000</v>
+      </c>
+      <c r="V32" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W32" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X32" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB32" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH32" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ32" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>45625.25</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>45625.75</v>
+      </c>
+      <c r="C33" t="n">
+        <v>7</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>8</v>
+      </c>
+      <c r="F33" t="n">
+        <v>12</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>period_2</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>WED01_LT01_3002</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J33" t="n">
+        <v>57867.84764285013</v>
+      </c>
+      <c r="K33" t="n">
+        <v>12000</v>
+      </c>
+      <c r="L33" t="n">
+        <v>45867.84764285013</v>
+      </c>
+      <c r="M33" t="n">
+        <v>55.15692796963216</v>
+      </c>
+      <c r="N33" t="n">
+        <v>9.041974529664218</v>
+      </c>
+      <c r="O33" t="n">
+        <v>3.905221911630801</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0.1058272675262239</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0.1531603422776934</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="S33" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T33" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U33" t="n">
+        <v>36000</v>
+      </c>
+      <c r="V33" t="n">
+        <v>3000</v>
+      </c>
+      <c r="W33" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X33" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>6.446125800106699</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>3.191577303789015</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>0.1328034132773035</v>
+      </c>
+      <c r="AB33" t="n">
+        <v>0.07718485044495821</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH33" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ33" t="n">
+        <v>100</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL33" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>